<commit_message>
fix: repair XLSX table/header/merged structure + styles (P0)
Fixture:
- Table ref A1:D2 (data only), merge A3:D3 (outside table)
- Header row: Column1-4 strings (matches tableColumns)
- Data row: formula/boolean/number/error cell types
- Conditional formatting sqref=C2 (data row)

Exporter:
- XLSX_STYLES: add cellStyles (Normal, builtinId=0), tableStyles,
  font family/scheme, border children, font sz/name
- This fixes 'Workbook contains no default style' warning from openpyxl

Updated SHA-256 hash for regenerated XLSX fixture
Fidelity-check passes all 4 cases
8 package_export tests pass
</commit_message>
<xml_diff>
--- a/fidelity/fixtures/workbook-rich.xlsx
+++ b/fidelity/fixtures/workbook-rich.xlsx
@@ -13,6 +13,8 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -24,7 +26,13 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -32,6 +40,10 @@
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -56,8 +68,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FidelityTable" displayName="FidelityTable" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FidelityTable" displayName="FidelityTable" ref="A1:D2" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:D2"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Column1"/>
     <tableColumn id="2" name="Column2"/>
@@ -78,30 +90,45 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Workbook Fidelity</t>
+          <t>Column1</t>
         </is>
       </c>
-      <c r="B1" t="b">
-        <v>1</v>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Column2</t>
+        </is>
       </c>
-      <c r="C1" t="n">
-        <v>42</v>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Column3</t>
+        </is>
       </c>
-      <c r="D1" t="e">
-        <v>#N/A</v>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Column4</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2">
-        <f>SUM(C1,8)</f>
+        <f>SUM(C2,8)</f>
         <v>50</v>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D2" t="e">
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A3:D3"/>
   </mergeCells>
-  <conditionalFormatting sqref="C1">
+  <conditionalFormatting sqref="C2">
     <cfRule type="cellIs" priority="1" operator="greaterThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>